<commit_message>
Update templates, add tests
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Schema" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Context" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Predicates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Classes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Units" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Extra" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Context" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Predicates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Classes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Units" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,9 @@
     <font>
       <b val="1"/>
       <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <sz val="11"/>
     </font>
   </fonts>
@@ -103,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -151,6 +155,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4320,6 +4326,238 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="74" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Include this info (yes/no) Test becomes root object, not cell</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Example dataset title</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>What the dataset contains, and anything needed to read it correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>coincell</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>battery</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Publisher</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>License</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://creativecommons.org/licenses/by/4.0/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Date issued</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Date published</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Publication DOI</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1234/example.2026.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Dataset URL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5281/zenodo.1234567</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Dataset API URL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/api/records/1234567</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Citation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>F. Lastname et al., Example Journal 1, 100 (2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Figures</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fig. 1a</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fig. 2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Authors</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Affiliations</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Firstname Lastname</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Corsin Battaglia</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4428,7 +4666,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4653,13 +4891,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4800,164 +5038,188 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Customcells</t>
+          <t>EPFL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q120784603</t>
+          <t>https://www.wikidata.org/wiki/Q262760</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Solvionic</t>
+          <t>ETH Zurich</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q30285492</t>
+          <t>https://www.wikidata.org/wiki/Q11942</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Celgard</t>
+          <t>Customcells</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q122199856</t>
+          <t>https://www.wikidata.org/wiki/Q120784603</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Hohsen</t>
+          <t>Solvionic</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q138027768</t>
+          <t>https://www.wikidata.org/wiki/Q30285492</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Corsin Battaglia</t>
+          <t>Celgard</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://orcid.org/0000-0002-5003-1134</t>
+          <t>https://www.wikidata.org/wiki/Q122199856</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nukorn Plainpan</t>
+          <t>Hohsen</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://orcid.org/0009-0002-6447-8057</t>
+          <t>https://www.wikidata.org/wiki/Q138027768</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Graham Kimbell</t>
+          <t>Corsin Battaglia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://orcid.org/0000-0001-9610-3589</t>
+          <t>https://orcid.org/0000-0002-5003-1134</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Enea Svaluto-Ferro</t>
+          <t>Nukorn Plainpan</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://orcid.org/0009-0004-4673-7806</t>
+          <t>https://orcid.org/0009-0002-6447-8057</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R2032</t>
+          <t>Graham Kimbell</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0001-9610-3589</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ElectrochemicalHalfCell</t>
+          <t>Enea Svaluto-Ferro</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0009-0004-4673-7806</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CarbonBlack</t>
+          <t>R2032</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>StainlessSteel</t>
+          <t>ElectrochemicalHalfCell</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Polypropylene</t>
+          <t>CarbonBlack</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>StainlessSteel</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CarboxymethylCellulose</t>
+          <t>Polypropylene</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>StyreneButadiene</t>
+          <t>Lithium</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FluoroethyleneCarbonate</t>
+          <t>CarboxymethylCellulose</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
+        <is>
+          <t>StyreneButadiene</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>FluoroethyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>GlassFibreSeparator</t>
         </is>
@@ -4968,7 +5230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Update coincell template electrolyte vol
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -4194,7 +4194,7 @@
         </is>
       </c>
       <c r="B148" s="5" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>CellCan, NegativeElectrode, Separator, 100.0 uL Electrolyte, PositiveElectrode, 1.0 mm Spacer, Spring, CellLid</t>
+          <t>CellCan, NegativeElectrode, Separator, 30.0 uL Electrolyte, PositiveElectrode, 1.0 mm Spacer, Spring, CellLid</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Update coincell template electrolyte vol (#100)
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -4194,7 +4194,7 @@
         </is>
       </c>
       <c r="B148" s="5" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>CellCan, NegativeElectrode, Separator, 100.0 uL Electrolyte, PositiveElectrode, 1.0 mm Spacer, Spring, CellLid</t>
+          <t>CellCan, NegativeElectrode, Separator, 30.0 uL Electrolyte, PositiveElectrode, 1.0 mm Spacer, Spring, CellLid</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Update extras (-> references) sheet
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Schema" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Extra" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@References" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Context" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Predicates" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Classes" sheetId="5" state="visible" r:id="rId5"/>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,9 +41,6 @@
     <font>
       <b val="1"/>
       <i val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <sz val="11"/>
     </font>
   </fonts>
@@ -107,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -155,8 +152,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -869,7 +864,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1.1.18</t>
+          <t>1.2.0</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -4326,224 +4321,619 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="74" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>Include this info (yes/no) Test becomes root object</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>No</t>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>References</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Example dataset title</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Include references in metadata file (yes/no)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>What the dataset contains, and anything needed to read it correctly.</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>References for dataset</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>Keywords</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>coincell</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>battery</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Dataset name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Dataset for publication "Toward an autonomous robotic battery materials research platform powered by automated workflow and ontologized findable, accessible, interoperable, and reusable data management"</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Dataset description</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>This dataset comprises detailed data from 199 coin cell batteries featuring either NMC//graphite or LFP//graphite chemistries cycled for 1000 cycles. All batteries were assembled and cycled using the automated robotic battery materials research platform, Aurora, at Empa, the Swiss Federal Laboratories for Materials Science and Technology, within the Laboratory for Materials for Energy Conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Dataset publisher</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Empa</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>License</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Dataset license</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>https://creativecommons.org/licenses/by/4.0/</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>Date issued</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Date published</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Dataset date issued</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Publication DOI</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1234/example.2026.001</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Dataset date published</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Dataset URL</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.5281/zenodo.1234567</t>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5281/zenodo.15481956</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Dataset API URL</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://zenodo.org/api/records/1234567</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/api/records/15481956</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Citation</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>F. Lastname et al., Example Journal 1, 100 (2026).</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorA</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Enea Svaluto-Ferro</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>Figures</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorB</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Graham Kimbell</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorC</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>YeonJu Kim</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorD</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Nukorn Plainpan</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorE</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Benjamin Kunz</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorF</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Lina Schulz</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorG</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Raphael Läubli</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorH</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Maximilian Becker</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorI</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>David Reber</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorJ</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Peter Kraus</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorK</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Ruben-Simon Kühnel</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorL</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Corsin Battaglia</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>References for associated publications</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication DOI</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/batt.202500155</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication title</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Toward an Autonomous Robotic Battery Materials Research Platform Powered by Automated Workflow and Ontologized Findable, Accessible, Interoperable, and Reusable Data Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication figures</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Fig. 1a</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Fig. 2b</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>Authors</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>Affiliations</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Firstname Lastname</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorA</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Enea Svaluto-Ferro</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Empa</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorB</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Graham Kimbell</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorC</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>YeonJu Kim</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorD</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Nukorn Plainpan</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorE</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Benjamin Kunz</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorF</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Lina Schulz</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorG</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Raphael Läubli</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorH</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Maximilian Becker</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorI</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>David Reber</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorJ</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Peter Kraus</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorK</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Ruben-Simon Kühnel</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorL</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Corsin Battaglia</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Empa</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>EPFL</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>ETH Zurich</t>
         </is>
       </c>
     </row>
@@ -4897,7 +5287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5158,68 +5548,116 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R2032</t>
+          <t>YeonJu Kim</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0003-3024-6370</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ElectrochemicalHalfCell</t>
+          <t>David Reber</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-4426-8717</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CarbonBlack</t>
+          <t>Peter Kraus</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-4359-5003</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>StainlessSteel</t>
+          <t>Ruben-Simon Kühnel</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0003-1542-2970</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Polypropylene</t>
+          <t>R2032</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>ElectrochemicalHalfCell</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CarboxymethylCellulose</t>
+          <t>CarbonBlack</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>StyreneButadiene</t>
+          <t>StainlessSteel</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>FluoroethyleneCarbonate</t>
+          <t>Polypropylene</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
+        <is>
+          <t>Lithium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CarboxymethylCellulose</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>StyreneButadiene</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FluoroethyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>GlassFibreSeparator</t>
         </is>

</xml_diff>

<commit_message>
Update templates with more example classes
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -584,11 +584,7 @@
           <t>CoinCell</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C3" s="4" t="n"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -616,11 +612,7 @@
           <t>empa__ccid_123456</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -648,11 +640,7 @@
           <t>240616_bco_gr-NMC_01</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -680,11 +668,7 @@
           <t>2024-06-16</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -712,11 +696,7 @@
           <t>Empa</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -744,11 +724,7 @@
           <t>Corsin Battaglia</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -776,11 +752,7 @@
           <t>Battery2030+/PREMISE</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -804,11 +776,7 @@
           <t>manually</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -836,11 +804,7 @@
           <t>CoinCellSchema</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -868,11 +832,7 @@
           <t>1.2.0</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -912,11 +872,7 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -966,11 +922,7 @@
           <t>LithiumNickelManganeseCobaltOxide</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -994,11 +946,7 @@
           <t>LiNi0.6Mn0.2Co0.2O2</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -1048,11 +996,7 @@
           <t>PolyvinylideneFluoride</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="inlineStr">
         <is>
           <t>required</t>
@@ -1102,11 +1046,7 @@
           <t>CarbonBlack</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="inlineStr">
         <is>
           <t>required</t>
@@ -1310,11 +1250,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C30" s="4" t="n"/>
       <c r="D30" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1338,11 +1274,7 @@
           <t>Lithium</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1664,11 +1596,7 @@
           <t>Customcells</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C44" s="4" t="n"/>
       <c r="D44" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1690,11 +1618,7 @@
       <c r="B45" s="8" t="n">
         <v>100000030</v>
       </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C45" s="8" t="n"/>
       <c r="D45" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1714,11 +1638,7 @@
         </is>
       </c>
       <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C46" s="4" t="n"/>
       <c r="D46" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1738,11 +1658,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C47" s="8" t="n"/>
       <c r="D47" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1762,11 +1678,7 @@
         </is>
       </c>
       <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C48" s="4" t="n"/>
       <c r="D48" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1786,11 +1698,7 @@
         </is>
       </c>
       <c r="B49" s="8" t="n"/>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C49" s="8" t="n"/>
       <c r="D49" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1810,11 +1718,7 @@
         </is>
       </c>
       <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1834,11 +1738,7 @@
         </is>
       </c>
       <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1858,11 +1758,7 @@
         </is>
       </c>
       <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1882,11 +1778,7 @@
         </is>
       </c>
       <c r="B53" s="8" t="n"/>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1922,11 +1814,7 @@
           <t>Copper</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C55" s="4" t="n"/>
       <c r="D55" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -1976,11 +1864,7 @@
           <t>Graphite</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C57" s="4" t="n"/>
       <c r="D57" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2030,11 +1914,7 @@
           <t>PolyvinylideneFluoride</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2084,11 +1964,7 @@
           <t>CarbonBlack</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2292,11 +2168,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C70" s="4" t="n"/>
       <c r="D70" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2320,11 +2192,7 @@
           <t>Lithium</t>
         </is>
       </c>
-      <c r="C71" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C71" s="12" t="n"/>
       <c r="D71" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2646,11 +2514,7 @@
           <t>Customcells</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C84" s="4" t="n"/>
       <c r="D84" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2674,11 +2538,7 @@
           <t>11113, A-1594</t>
         </is>
       </c>
-      <c r="C85" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C85" s="12" t="n"/>
       <c r="D85" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2698,11 +2558,7 @@
         </is>
       </c>
       <c r="B86" s="4" t="n"/>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C86" s="4" t="n"/>
       <c r="D86" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2722,11 +2578,7 @@
         </is>
       </c>
       <c r="B87" s="12" t="n"/>
-      <c r="C87" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C87" s="12" t="n"/>
       <c r="D87" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2746,11 +2598,7 @@
         </is>
       </c>
       <c r="B88" s="4" t="n"/>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C88" s="4" t="n"/>
       <c r="D88" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2770,11 +2618,7 @@
         </is>
       </c>
       <c r="B89" s="12" t="n"/>
-      <c r="C89" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C89" s="12" t="n"/>
       <c r="D89" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2794,11 +2638,7 @@
         </is>
       </c>
       <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C90" s="4" t="n"/>
       <c r="D90" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2818,11 +2658,7 @@
         </is>
       </c>
       <c r="B91" s="12" t="n"/>
-      <c r="C91" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C91" s="12" t="n"/>
       <c r="D91" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2842,11 +2678,7 @@
         </is>
       </c>
       <c r="B92" s="4" t="n"/>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C92" s="4" t="n"/>
       <c r="D92" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2866,11 +2698,7 @@
         </is>
       </c>
       <c r="B93" s="12" t="n"/>
-      <c r="C93" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C93" s="12" t="n"/>
       <c r="D93" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2906,11 +2734,7 @@
           <t>EthyleneCarbonate</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C95" s="4" t="n"/>
       <c r="D95" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2960,11 +2784,7 @@
           <t>EthylMethylCarbonate</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C97" s="4" t="n"/>
       <c r="D97" s="4" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -3014,11 +2834,7 @@
           <t>LithiumHexafluorophosphate</t>
         </is>
       </c>
-      <c r="C99" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C99" s="4" t="n"/>
       <c r="D99" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3068,11 +2884,7 @@
           <t>LithiumBisfluorosulfonylimide</t>
         </is>
       </c>
-      <c r="C101" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C101" s="4" t="n"/>
       <c r="D101" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3122,11 +2934,7 @@
           <t>VinyleneCarbonate</t>
         </is>
       </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C103" s="4" t="n"/>
       <c r="D103" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3176,11 +2984,7 @@
           <t>TrisTrimethylsilyPhosphite</t>
         </is>
       </c>
-      <c r="C105" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C105" s="4" t="n"/>
       <c r="D105" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3358,11 +3162,7 @@
           <t>Solvionic</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C113" s="4" t="n"/>
       <c r="D113" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3382,11 +3182,7 @@
         </is>
       </c>
       <c r="B114" s="16" t="n"/>
-      <c r="C114" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C114" s="16" t="n"/>
       <c r="D114" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3406,11 +3202,7 @@
         </is>
       </c>
       <c r="B115" s="4" t="n"/>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C115" s="4" t="n"/>
       <c r="D115" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3430,11 +3222,7 @@
         </is>
       </c>
       <c r="B116" s="16" t="n"/>
-      <c r="C116" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C116" s="16" t="n"/>
       <c r="D116" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3454,11 +3242,7 @@
         </is>
       </c>
       <c r="B117" s="4" t="n"/>
-      <c r="C117" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C117" s="4" t="n"/>
       <c r="D117" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3478,11 +3262,7 @@
         </is>
       </c>
       <c r="B118" s="16" t="n"/>
-      <c r="C118" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C118" s="16" t="n"/>
       <c r="D118" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3502,11 +3282,7 @@
         </is>
       </c>
       <c r="B119" s="4" t="n"/>
-      <c r="C119" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C119" s="4" t="n"/>
       <c r="D119" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3526,11 +3302,7 @@
         </is>
       </c>
       <c r="B120" s="16" t="n"/>
-      <c r="C120" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C120" s="16" t="n"/>
       <c r="D120" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3550,11 +3322,7 @@
         </is>
       </c>
       <c r="B121" s="4" t="n"/>
-      <c r="C121" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C121" s="4" t="n"/>
       <c r="D121" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3574,11 +3342,7 @@
         </is>
       </c>
       <c r="B122" s="16" t="n"/>
-      <c r="C122" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C122" s="16" t="n"/>
       <c r="D122" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3598,11 +3362,7 @@
         </is>
       </c>
       <c r="B123" s="4" t="n"/>
-      <c r="C123" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C123" s="4" t="n"/>
       <c r="D123" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3622,11 +3382,7 @@
         </is>
       </c>
       <c r="B124" s="16" t="n"/>
-      <c r="C124" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C124" s="16" t="n"/>
       <c r="D124" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3646,11 +3402,7 @@
         </is>
       </c>
       <c r="B125" s="4" t="n"/>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C125" s="4" t="n"/>
       <c r="D125" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3670,11 +3422,7 @@
         </is>
       </c>
       <c r="B126" s="16" t="n"/>
-      <c r="C126" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C126" s="16" t="n"/>
       <c r="D126" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3710,11 +3458,7 @@
           <t>Polypropylene</t>
         </is>
       </c>
-      <c r="C128" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C128" s="4" t="n"/>
       <c r="D128" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3840,11 +3584,7 @@
           <t>Celgard</t>
         </is>
       </c>
-      <c r="C134" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C134" s="4" t="n"/>
       <c r="D134" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3866,11 +3606,7 @@
       <c r="B135" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="C135" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C135" s="5" t="n"/>
       <c r="D135" s="5" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3906,11 +3642,7 @@
           <t>R2032</t>
         </is>
       </c>
-      <c r="C137" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C137" s="4" t="n"/>
       <c r="D137" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3934,11 +3666,7 @@
           <t>StainlessSteel</t>
         </is>
       </c>
-      <c r="C138" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C138" s="5" t="n"/>
       <c r="D138" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -3962,11 +3690,7 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C139" s="4" t="n"/>
       <c r="D139" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3990,11 +3714,7 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C140" s="5" t="n"/>
       <c r="D140" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -4226,11 +3946,7 @@
           <t>CellCan, NegativeElectrode, Separator, 30.0 uL Electrolyte, PositiveElectrode, 1.0 mm Spacer, Spring, CellLid</t>
         </is>
       </c>
-      <c r="C149" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C149" s="4" t="n"/>
       <c r="D149" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -4266,11 +3982,7 @@
           <t>Hohsen</t>
         </is>
       </c>
-      <c r="C151" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C151" s="4" t="n"/>
       <c r="D151" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -4294,11 +4006,7 @@
           <t>2032, SUS316L</t>
         </is>
       </c>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C152" s="5" t="n"/>
       <c r="D152" s="5" t="inlineStr">
         <is>
           <t>optional</t>
@@ -5035,22 +4743,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Term</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>IRI</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
@@ -5152,20 +4866,20 @@
   <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Predicate</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>Default class</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -5404,7 +5118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5426,164 +5140,528 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>CoinCell</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Classes available to the @Schema sheet Value column. Classes must already exist in the ontology. You can declare your own custom classes in the @Context sheet. This column is a reference list, a value already known to the ontology works even if it is not listed.</t>
+          <t>Cell and case. Classes available to the @Schema sheet Value column. Classes must already exist in the ontology. You can declare your own custom classes in the @Context sheet. This column is a reference list, a value already known to the ontology works even if it is not listed.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>R2032</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LithiumNickelManganeseCobaltOxide</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://pubchem.ncbi.nlm.nih.gov/substance/485083898</t>
+          <t>R2025</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Graphite</t>
+          <t>R2016</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PolyvinylideneFluoride</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CarbonBlack</t>
-        </is>
-      </c>
-    </row>
+          <t>ElectrochemicalHalfCell</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EthyleneCarbonate</t>
+          <t>LithiumNickelManganeseCobaltOxide</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Positive electrode active materials.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EthylMethylCarbonate</t>
+          <t>LithiumNickelManganeseCobaltOxide111</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LithiumHexafluorophosphate</t>
+          <t>LithiumNickelManganeseCobaltOxide532</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VinyleneCarbonate</t>
+          <t>LithiumNickelManganeseCobaltOxide622</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LithiumBisfluorosulfonylimide</t>
+          <t>LithiumNickelManganeseCobaltOxide811</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TrisTrimethylsilyPhosphite</t>
+          <t>LithiumNickelCobaltAluminiumOxide</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Polyolefin</t>
+          <t>LithiumNickelManganeseOxide</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R2032</t>
+          <t>LithiumCobaltOxide</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ElectrochemicalHalfCell</t>
+          <t>LithiumManganeseOxide</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>StainlessSteel</t>
+          <t>LithiumIronPhosphate</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Polypropylene</t>
+          <t>LithiumManganeseIronPhosphate</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lithium</t>
+          <t>SodiumIronPhosphate</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CarboxymethylCellulose</t>
+          <t>SodiumManganeseOxide</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>StyreneButadiene</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>FluoroethyleneCarbonate</t>
-        </is>
-      </c>
-    </row>
+          <t>SodiumCobaltOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Graphite</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Negative electrode active materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HardCarbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SiliconGraphite</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Silicon</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SiliconOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SiliconMonoxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LithiumTitanate</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Lithium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Current collectors and other metals</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Nickel</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>StainlessSteel</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Titanium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PolyvinylideneFluoride</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Binders</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CarboxymethylCellulose</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>StyreneButadiene</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Polytetrafluoroethylene</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PolyacrylicAcid</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CarbonBlack</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Conductive additives</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Graphene</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>EthyleneCarbonate</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Electrolyte solvents</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>EthylMethylCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DimethylCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DiethylCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PropyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Dimethoxyethane</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Dioxolane</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Sulfolane</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>LithiumHexafluorophosphate</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Electrolyte salts</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LithiumBisfluorosulfonylimide</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LithiumBistrifluoromethanesulfonylimide</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>LithiumTetrafluoroborate</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>LithiumPerchlorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>LithiumBisoxalatoborate</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>LithiumDifluorooxalatoborate</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>LithiumTriflate</t>
+        </is>
+      </c>
+    </row>
+    <row r="65"/>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>FluoroethyleneCarbonate</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Electrolyte additives</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>VinyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>VinylEthyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>TrisTrimethylsilyPhosphite</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Polypropylene</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Separators and separator coatings</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Polyethylene</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Polyolefin</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>GlassFibreSeparator</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>PorousSeparator</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CeramicCoating</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>AluminiumOxide</t>
         </is>
       </c>
     </row>
@@ -5602,7 +5680,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="74" customWidth="1" min="4" max="4"/>
   </cols>
@@ -5615,7 +5693,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -5895,22 +5973,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>Unit class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New sheet/column layout (#101)
Adds "@References" sheet for publication, dataset, author info
Splits "@Classes" into "@Individuals" sheet for people, organisations
Update column names in all sheets
Adds multiple output types to app
More flexible sheet/column discovery
Remove "No Unit" requirement
Fix notes/documentation
All organisation IRIs fixed and use wikidata entity
Allow custom classes, namespaces in context
More tests and bugfixes

Converter is backwards compatible, new sheets are not
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Schema" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Context" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Predicates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Classes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Units" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@References" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Context" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Predicates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Classes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Individuals" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="@Units" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -550,7 +552,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -582,11 +584,7 @@
           <t>CoinCell</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C3" s="4" t="n"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -614,11 +612,7 @@
           <t>empa__ccid_123456</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -646,11 +640,7 @@
           <t>240616_bco_gr-NMC_01</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -678,11 +668,7 @@
           <t>2024-06-16</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -710,11 +696,7 @@
           <t>Empa</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -722,7 +704,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Organisation that made the cell, value should be in @classes with ID</t>
+          <t>Organisation that made the cell. List it in @Individuals to give it an IRI.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -742,11 +724,7 @@
           <t>Corsin Battaglia</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -754,7 +732,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Person that made the cell, value should be in @classes with ID</t>
+          <t>Person that made the cell. List them in @Individuals to give them an ORCID.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -774,11 +752,7 @@
           <t>Battery2030+/PREMISE</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -802,11 +776,7 @@
           <t>manually</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -834,11 +804,7 @@
           <t>CoinCellSchema</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -863,14 +829,10 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1.1.18</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+          <t>2.0.0</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -910,11 +872,7 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -964,11 +922,7 @@
           <t>LithiumNickelManganeseCobaltOxide</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -992,11 +946,7 @@
           <t>LiNi0.6Mn0.2Co0.2O2</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -1046,11 +996,7 @@
           <t>PolyvinylideneFluoride</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="inlineStr">
         <is>
           <t>required</t>
@@ -1100,11 +1046,7 @@
           <t>CarbonBlack</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="inlineStr">
         <is>
           <t>required</t>
@@ -1308,11 +1250,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C30" s="4" t="n"/>
       <c r="D30" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1336,11 +1274,7 @@
           <t>Lithium</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1662,11 +1596,7 @@
           <t>Customcells</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C44" s="4" t="n"/>
       <c r="D44" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1688,11 +1618,7 @@
       <c r="B45" s="8" t="n">
         <v>100000030</v>
       </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C45" s="8" t="n"/>
       <c r="D45" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1712,11 +1638,7 @@
         </is>
       </c>
       <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C46" s="4" t="n"/>
       <c r="D46" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1736,11 +1658,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C47" s="8" t="n"/>
       <c r="D47" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1760,11 +1678,7 @@
         </is>
       </c>
       <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C48" s="4" t="n"/>
       <c r="D48" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1784,11 +1698,7 @@
         </is>
       </c>
       <c r="B49" s="8" t="n"/>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C49" s="8" t="n"/>
       <c r="D49" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1808,11 +1718,7 @@
         </is>
       </c>
       <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1832,11 +1738,7 @@
         </is>
       </c>
       <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1856,11 +1758,7 @@
         </is>
       </c>
       <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1880,11 +1778,7 @@
         </is>
       </c>
       <c r="B53" s="8" t="n"/>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="inlineStr">
         <is>
           <t>optional</t>
@@ -1920,11 +1814,7 @@
           <t>Copper</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C55" s="4" t="n"/>
       <c r="D55" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -1974,11 +1864,7 @@
           <t>Graphite</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C57" s="4" t="n"/>
       <c r="D57" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2028,11 +1914,7 @@
           <t>PolyvinylideneFluoride</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2082,11 +1964,7 @@
           <t>CarbonBlack</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2290,11 +2168,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C70" s="4" t="n"/>
       <c r="D70" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2318,11 +2192,7 @@
           <t>Lithium</t>
         </is>
       </c>
-      <c r="C71" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C71" s="12" t="n"/>
       <c r="D71" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2644,11 +2514,7 @@
           <t>Customcells</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C84" s="4" t="n"/>
       <c r="D84" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2672,11 +2538,7 @@
           <t>11113, A-1594</t>
         </is>
       </c>
-      <c r="C85" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C85" s="12" t="n"/>
       <c r="D85" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2696,11 +2558,7 @@
         </is>
       </c>
       <c r="B86" s="4" t="n"/>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C86" s="4" t="n"/>
       <c r="D86" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2720,11 +2578,7 @@
         </is>
       </c>
       <c r="B87" s="12" t="n"/>
-      <c r="C87" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C87" s="12" t="n"/>
       <c r="D87" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2744,11 +2598,7 @@
         </is>
       </c>
       <c r="B88" s="4" t="n"/>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C88" s="4" t="n"/>
       <c r="D88" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2768,11 +2618,7 @@
         </is>
       </c>
       <c r="B89" s="12" t="n"/>
-      <c r="C89" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C89" s="12" t="n"/>
       <c r="D89" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2792,11 +2638,7 @@
         </is>
       </c>
       <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C90" s="4" t="n"/>
       <c r="D90" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2816,11 +2658,7 @@
         </is>
       </c>
       <c r="B91" s="12" t="n"/>
-      <c r="C91" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C91" s="12" t="n"/>
       <c r="D91" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2840,11 +2678,7 @@
         </is>
       </c>
       <c r="B92" s="4" t="n"/>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C92" s="4" t="n"/>
       <c r="D92" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2864,11 +2698,7 @@
         </is>
       </c>
       <c r="B93" s="12" t="n"/>
-      <c r="C93" s="12" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C93" s="12" t="n"/>
       <c r="D93" s="12" t="inlineStr">
         <is>
           <t>optional</t>
@@ -2904,11 +2734,7 @@
           <t>EthyleneCarbonate</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C95" s="4" t="n"/>
       <c r="D95" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -2958,11 +2784,7 @@
           <t>EthylMethylCarbonate</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C97" s="4" t="n"/>
       <c r="D97" s="4" t="inlineStr">
         <is>
           <t>recommended</t>
@@ -3012,11 +2834,7 @@
           <t>LithiumHexafluorophosphate</t>
         </is>
       </c>
-      <c r="C99" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C99" s="4" t="n"/>
       <c r="D99" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3066,11 +2884,7 @@
           <t>LithiumBisfluorosulfonylimide</t>
         </is>
       </c>
-      <c r="C101" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C101" s="4" t="n"/>
       <c r="D101" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3120,11 +2934,7 @@
           <t>VinyleneCarbonate</t>
         </is>
       </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C103" s="4" t="n"/>
       <c r="D103" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3174,11 +2984,7 @@
           <t>TrisTrimethylsilyPhosphite</t>
         </is>
       </c>
-      <c r="C105" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C105" s="4" t="n"/>
       <c r="D105" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3356,11 +3162,7 @@
           <t>Solvionic</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C113" s="4" t="n"/>
       <c r="D113" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3380,11 +3182,7 @@
         </is>
       </c>
       <c r="B114" s="16" t="n"/>
-      <c r="C114" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C114" s="16" t="n"/>
       <c r="D114" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3404,11 +3202,7 @@
         </is>
       </c>
       <c r="B115" s="4" t="n"/>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C115" s="4" t="n"/>
       <c r="D115" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3428,11 +3222,7 @@
         </is>
       </c>
       <c r="B116" s="16" t="n"/>
-      <c r="C116" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C116" s="16" t="n"/>
       <c r="D116" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3452,11 +3242,7 @@
         </is>
       </c>
       <c r="B117" s="4" t="n"/>
-      <c r="C117" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C117" s="4" t="n"/>
       <c r="D117" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3476,11 +3262,7 @@
         </is>
       </c>
       <c r="B118" s="16" t="n"/>
-      <c r="C118" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C118" s="16" t="n"/>
       <c r="D118" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3500,11 +3282,7 @@
         </is>
       </c>
       <c r="B119" s="4" t="n"/>
-      <c r="C119" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C119" s="4" t="n"/>
       <c r="D119" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3524,11 +3302,7 @@
         </is>
       </c>
       <c r="B120" s="16" t="n"/>
-      <c r="C120" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C120" s="16" t="n"/>
       <c r="D120" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3548,11 +3322,7 @@
         </is>
       </c>
       <c r="B121" s="4" t="n"/>
-      <c r="C121" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C121" s="4" t="n"/>
       <c r="D121" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3572,11 +3342,7 @@
         </is>
       </c>
       <c r="B122" s="16" t="n"/>
-      <c r="C122" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C122" s="16" t="n"/>
       <c r="D122" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3596,11 +3362,7 @@
         </is>
       </c>
       <c r="B123" s="4" t="n"/>
-      <c r="C123" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C123" s="4" t="n"/>
       <c r="D123" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3620,11 +3382,7 @@
         </is>
       </c>
       <c r="B124" s="16" t="n"/>
-      <c r="C124" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C124" s="16" t="n"/>
       <c r="D124" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3644,11 +3402,7 @@
         </is>
       </c>
       <c r="B125" s="4" t="n"/>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C125" s="4" t="n"/>
       <c r="D125" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3668,11 +3422,7 @@
         </is>
       </c>
       <c r="B126" s="16" t="n"/>
-      <c r="C126" s="16" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C126" s="16" t="n"/>
       <c r="D126" s="16" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3708,11 +3458,7 @@
           <t>Polypropylene</t>
         </is>
       </c>
-      <c r="C128" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C128" s="4" t="n"/>
       <c r="D128" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3838,11 +3584,7 @@
           <t>Celgard</t>
         </is>
       </c>
-      <c r="C134" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C134" s="4" t="n"/>
       <c r="D134" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3864,11 +3606,7 @@
       <c r="B135" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="C135" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C135" s="5" t="n"/>
       <c r="D135" s="5" t="inlineStr">
         <is>
           <t>optional</t>
@@ -3904,11 +3642,7 @@
           <t>R2032</t>
         </is>
       </c>
-      <c r="C137" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C137" s="4" t="n"/>
       <c r="D137" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3932,11 +3666,7 @@
           <t>StainlessSteel</t>
         </is>
       </c>
-      <c r="C138" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C138" s="5" t="n"/>
       <c r="D138" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -3960,11 +3690,7 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C139" s="4" t="n"/>
       <c r="D139" s="4" t="inlineStr">
         <is>
           <t>required</t>
@@ -3988,11 +3714,7 @@
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C140" s="5" t="n"/>
       <c r="D140" s="5" t="inlineStr">
         <is>
           <t>required</t>
@@ -4224,11 +3946,7 @@
           <t>CellCan, NegativeElectrode, Separator, 30.0 uL Electrolyte, PositiveElectrode, 1.0 mm Spacer, Spring, CellLid</t>
         </is>
       </c>
-      <c r="C149" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C149" s="4" t="n"/>
       <c r="D149" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -4264,11 +3982,7 @@
           <t>Hohsen</t>
         </is>
       </c>
-      <c r="C151" s="4" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C151" s="4" t="n"/>
       <c r="D151" s="4" t="inlineStr">
         <is>
           <t>optional</t>
@@ -4292,11 +4006,7 @@
           <t>2032, SUS316L</t>
         </is>
       </c>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>No Unit</t>
-        </is>
-      </c>
+      <c r="C152" s="5" t="n"/>
       <c r="D152" s="5" t="inlineStr">
         <is>
           <t>optional</t>
@@ -4320,106 +4030,715 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Metadata</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Extra values  -&gt;  affiliations for an author, a description for a data file, or more items for a list</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://schema.org/</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Include references in metadata file (yes/no)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>emmo</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://w3id.org/emmo#</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>References for dataset</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>echem</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://w3id.org/emmo/domain/electrochemistry#</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Dataset name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Dataset for publication "Toward an autonomous robotic battery materials research platform powered by automated workflow and ontologized findable, accessible, interoperable, and reusable data management"</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>battery</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://w3id.org/emmo/domain/battery#</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Dataset description</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>This dataset comprises detailed data from 199 coin cell batteries featuring either NMC//graphite or LFP//graphite chemistries cycled for 1000 cycles. All batteries were assembled and cycled using the automated robotic battery materials research platform, Aurora, at Empa, the Swiss Federal Laboratories for Materials Science and Technology, within the Laboratory for Materials for Energy Conversion.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>chemical</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://w3id.org/emmo/domain/chemical-substance#</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Dataset publisher</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://qudt.org/vocab/unit/</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Dataset license</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>https://creativecommons.org/licenses/by/4.0/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>rdfs</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>http://www.w3.org/2000/01/rdf-schema#</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Dataset date issued</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Dataset date published</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Dataset URL</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5281/zenodo.15481956</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dataset API URL</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/api/records/15481956</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorA</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Enea Svaluto-Ferro</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorB</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Graham Kimbell</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorC</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>YeonJu Kim</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorD</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Nukorn Plainpan</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorE</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Benjamin Kunz</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorF</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Lina Schulz</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorG</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Raphael Läubli</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorH</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Maximilian Becker</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorI</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>David Reber</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorJ</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Peter Kraus</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorK</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Ruben-Simon Kühnel</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Dataset authorL</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Corsin Battaglia</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>References for associated publications</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication DOI</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/batt.202500155</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication title</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Toward an Autonomous Robotic Battery Materials Research Platform Powered by Automated Workflow and Ontologized Findable, Accessible, Interoperable, and Reusable Data Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication figures</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Fig. 1a</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Fig. 2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorA</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Enea Svaluto-Ferro</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorB</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Graham Kimbell</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorC</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>YeonJu Kim</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorD</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Nukorn Plainpan</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorE</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Benjamin Kunz</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorF</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Lina Schulz</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorG</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Raphael Läubli</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorH</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Maximilian Becker</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorI</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>David Reber</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorJ</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Peter Kraus</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorK</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Ruben-Simon Kühnel</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Associated publication authorL</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Corsin Battaglia</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>References for data files</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Data zip file</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Dataset-rocrate.zip</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Tabular data schema</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>https://w3id.org/battery-data-alliance/ontology/battery-data-format/schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Data fileA</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>empa__ccid000001/empa__ccid000001.bdf.parquet</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Time series electrochemical data as parquet with Battery Data Format columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Data fileB</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>empa__ccid000001/empa__ccid000001.bdf.csv</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Time series electrochemical data as csv with Battery Data Format columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Raw data fileA</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>empa__ccid000001/empa__ccid000001_GCPL_C01.mpr</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Raw cycling data, Biologic EC-Lab binary mpr format</t>
         </is>
       </c>
     </row>
@@ -4434,217 +4753,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Term</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>IRI</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hasActiveMaterial</t>
+          <t>schema</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://schema.org/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hasBinder</t>
+          <t>emmo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Binder</t>
+          <t>https://w3id.org/emmo#</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>hasCase</t>
+          <t>echem</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://w3id.org/emmo/domain/electrochemistry#</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>hasCoating</t>
+          <t>battery</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://w3id.org/emmo/domain/battery#</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>hasConductiveAdditive</t>
+          <t>chemical</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ConductiveAdditive</t>
+          <t>https://w3id.org/emmo/domain/chemical-substance#</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hasCurrentCollector</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CurrentCollector</t>
+          <t>https://qudt.org/vocab/unit/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>hasElectrolyte</t>
+          <t>rdfs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OrganicElectrolyte</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>hasNegativeElectrode</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Electrode</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>hasPositiveElectrode</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Electrode</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>hasSeparator</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Separator</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>hasSolute</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Solute</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>hasSolvent</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Solvent</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>hasConstituent</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>hasInput</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>hasProperty</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>hasMeasuredProperty</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>hasOutput</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hasReferenceElectrode</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>ReferenceElectrode</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>hasAdditive</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Additive</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>hasStringValue</t>
+          <t>http://www.w3.org/2000/01/rdf-schema#</t>
         </is>
       </c>
     </row>
@@ -4659,23 +4873,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="74" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Predicate</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Default class</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -4687,279 +4901,219 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aluminium</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>If the item is listed here without unique ID (e.g. R2032), this means the item is already ontologized in BattInFo ontology. No unique is required.</t>
+          <t>hasActiveMaterial</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ActiveMaterial</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>hasAdditive</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Additive</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LithiumNickelManganeseCobaltOxide</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://pubchem.ncbi.nlm.nih.gov/substance/485083898</t>
+          <t>hasBinder</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Binder</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Graphite</t>
+          <t>hasCoating</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Coating</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PolyvinylideneFluoride</t>
+          <t>hasConductiveAdditive</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ConductiveAdditive</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CarbonBlack</t>
+          <t>hasCurrentCollector</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CurrentCollector</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EthyleneCarbonate</t>
+          <t>hasElectrolyte</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Electrolyte</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EthylMethylCarbonate</t>
+          <t>hasNegativeElectrode</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NegativeElectrode</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LithiumHexafluorophosphate</t>
+          <t>hasPositiveElectrode</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PositiveElectrode</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>VinyleneCarbonate</t>
+          <t>hasReferenceElectrode</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ReferenceElectrode</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LithiumBisfluorosulfonylimide</t>
+          <t>hasSeparator</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Separator</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TrisTrimethylsilyPhosphite</t>
+          <t>hasSolute</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Solute</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Polyolefin</t>
+          <t>hasSolvent</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Solvent</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Empa</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://www.wikidata.org/wiki/Q683116</t>
+          <t>hasCase</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Customcells</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://www.wikidata.org/wiki/Q120784603</t>
+          <t>hasComponent</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Solvionic</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://www.wikidata.org/wiki/Q30285492</t>
+          <t>hasConstituent</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Celgard</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://www.wikidata.org/wiki/Q122199856</t>
+          <t>hasDatum</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Hohsen</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://www.wikidata.org/wiki/Q138027768</t>
+          <t>hasInput</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Corsin Battaglia</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://orcid.org/0000-0002-5003-1134</t>
+          <t>hasMeasuredProperty</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nukorn Plainpan</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://orcid.org/0009-0002-6447-8057</t>
+          <t>hasOutput</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Graham Kimbell</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>https://orcid.org/0000-0001-9610-3589</t>
+          <t>hasProperty</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Enea Svaluto-Ferro</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>https://orcid.org/0009-0004-4673-7806</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>R2032</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ElectrochemicalHalfCell</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>CarbonBlack</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>StainlessSteel</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Polypropylene</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Lithium</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>CarboxymethylCellulose</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>StyreneButadiene</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>FluoroethyleneCarbonate</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>GlassFibreSeparator</t>
+          <t>hasStringValue</t>
         </is>
       </c>
     </row>
@@ -4974,22 +5128,883 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CoinCell</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cell and case. Classes available to the @Schema sheet Value column. Classes must already exist in the ontology. You can declare your own custom classes in the @Context sheet. This column is a reference list, a value already known to the ontology works even if it is not listed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R2032</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ElectrochemicalHalfCell</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LithiumNickelManganeseCobaltOxide</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Positive electrode active materials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LithiumNickelManganeseCobaltOxide111</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LithiumNickelManganeseCobaltOxide532</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LithiumNickelManganeseCobaltOxide622</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LithiumNickelManganeseCobaltOxide811</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LithiumNickelCobaltAluminiumOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LithiumNickelManganeseOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LithiumCobaltOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LithiumManganeseOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LithiumIronPhosphate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LithiumManganeseIronPhosphate</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SodiumIronPhosphate</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SodiumManganeseOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SodiumCobaltOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Graphite</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Negative electrode active materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HardCarbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SiliconGraphite</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Silicon</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SiliconOxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SiliconMonoxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LithiumTitanate</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Lithium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Current collectors and other metals</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Nickel</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>StainlessSteel</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Titanium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PolyvinylideneFluoride</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Binders</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CarboxymethylCellulose</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>StyreneButadiene</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Polytetrafluoroethylene</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PolyacrylicAcid</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CarbonBlack</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Conductive additives</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Graphene</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>EthyleneCarbonate</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Electrolyte solvents</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>EthylMethylCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DimethylCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DiethylCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PropyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Dimethoxyethane</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Dioxolane</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Sulfolane</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>LithiumHexafluorophosphate</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Electrolyte salts</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LithiumBisfluorosulfonylimide</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LithiumBistrifluoromethanesulfonylimide</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>LithiumTetrafluoroborate</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>LithiumPerchlorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>LithiumBisoxalatoborate</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>LithiumDifluorooxalatoborate</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>LithiumTriflate</t>
+        </is>
+      </c>
+    </row>
+    <row r="65"/>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>FluoroethyleneCarbonate</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Electrolyte additives</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>VinyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>VinylEthyleneCarbonate</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>TrisTrimethylsilyPhosphite</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Polypropylene</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Separators and separator coatings</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Polyethylene</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Polyolefin</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>GlassFibreSeparator</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>PorousSeparator</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CeramicCoating</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>AluminiumOxide</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>IRI</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Corsin Battaglia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-5003-1134</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nukorn Plainpan</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0009-0002-6447-8057</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Graham Kimbell</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0001-9610-3589</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Enea Svaluto-Ferro</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0009-0004-4673-7806</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>YeonJu Kim</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0003-3024-6370</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>David Reber</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-4426-8717</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Peter Kraus</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-4359-5003</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ruben-Simon Kühnel</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>schema:Person</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0003-1542-2970</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Empa</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>schema:ResearchOrganization</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q683116</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>schema:ResearchOrganization</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q262760</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>schema:ResearchOrganization</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q11942</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Customcells</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>schema:Organization</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q120784603</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Solvionic</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>schema:Organization</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q30285492</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Celgard</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>schema:Organization</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q122199856</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hohsen</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>schema:Organization</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>http://www.wikidata.org/entity/Q138782243</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unit class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add input files to references sheet
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -829,7 +829,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2.0.0</t>
+          <t>2.1.0</t>
         </is>
       </c>
       <c r="C12" s="5" t="n"/>
@@ -4030,7 +4030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="74" customWidth="1" min="1" max="1"/>
@@ -4739,6 +4739,23 @@
       <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Raw cycling data, Biologic EC-Lab binary mpr format</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Input fileA</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>empa__ccid000001/empa__ccid000001.mps</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Cycling protocol, Biologic EC-Lab settings file</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve metadata hasInputs/hasOutputs (#105)
Raw data files change from hasInput to hasOutput

Add rows for input files like mps settings, which go to hasInput

If the user gives a folder structure without a zip-name, warn and drop `@id`
You cannot upload folders to Zenodo, so the `@id` and url would certainly be wrong
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -829,7 +829,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2.0.0</t>
+          <t>2.1.0</t>
         </is>
       </c>
       <c r="C12" s="5" t="n"/>
@@ -4030,7 +4030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="74" customWidth="1" min="1" max="1"/>
@@ -4739,6 +4739,23 @@
       <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Raw cycling data, Biologic EC-Lab binary mpr format</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Input fileA</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>empa__ccid000001/empa__ccid000001.mps</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Cycling protocol, Biologic EC-Lab settings file</t>
         </is>
       </c>
     </row>

</xml_diff>